<commit_message>
create conjunction and weighted detectors
</commit_message>
<xml_diff>
--- a/testResults/recognizersResults.xlsx
+++ b/testResults/recognizersResults.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,6 +455,11 @@
           <t>trunkAngleRecognizer</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>kneesDownRecognizer</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
@@ -508,6 +513,16 @@
           <t>SCORE</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>SCORE</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -555,6 +570,14 @@
       <c r="K3" t="n">
         <v>54.43662183593101</v>
       </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>46.04792875721753</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -602,6 +625,14 @@
       <c r="K4" t="n">
         <v>81.73906474938507</v>
       </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>9.489553167227132</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -649,6 +680,14 @@
       <c r="K5" t="n">
         <v>89.0534831548038</v>
       </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>13.78509184311913</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -696,6 +735,14 @@
       <c r="K6" t="n">
         <v>41.47956296365606</v>
       </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>24.43904402883065</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -743,6 +790,14 @@
       <c r="K7" t="n">
         <v>98.16792202432266</v>
       </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>77.24937964607919</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -790,6 +845,14 @@
       <c r="K8" t="n">
         <v>86.4083474727166</v>
       </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>-24.38500818830445</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -837,6 +900,14 @@
       <c r="K9" t="n">
         <v>97.6376708583107</v>
       </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>75.61611830333837</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -884,6 +955,14 @@
       <c r="K10" t="n">
         <v>72.00726351141846</v>
       </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>10.80926725669039</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -931,6 +1010,14 @@
       <c r="K11" t="n">
         <v>88.12382013188308</v>
       </c>
+      <c r="L11" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>87.85292807833882</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -978,6 +1065,14 @@
       <c r="K12" t="n">
         <v>65.87991783411722</v>
       </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>-23.1109847217271</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1025,6 +1120,14 @@
       <c r="K13" t="n">
         <v>69.00092895871938</v>
       </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>12.17803939781761</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1072,6 +1175,14 @@
       <c r="K14" t="n">
         <v>91.52540074663487</v>
       </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>4.377009113168582</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1119,6 +1230,14 @@
       <c r="K15" t="n">
         <v>49.15525932287592</v>
       </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>16.43977913192763</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1166,6 +1285,14 @@
       <c r="K16" t="n">
         <v>14.22705767821495</v>
       </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>9.345067540693298</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1213,6 +1340,14 @@
       <c r="K17" t="n">
         <v>2.609290858294099</v>
       </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>83.01624438438321</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1260,6 +1395,14 @@
       <c r="K18" t="n">
         <v>51.58539717753479</v>
       </c>
+      <c r="L18" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>29.95240519021135</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1307,6 +1450,14 @@
       <c r="K19" t="n">
         <v>17.50931995130208</v>
       </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>97.70309957445166</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1354,6 +1505,14 @@
       <c r="K20" t="n">
         <v>17.712211108605</v>
       </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>96.05048371238728</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1401,6 +1560,14 @@
       <c r="K21" t="n">
         <v>12.36876507368786</v>
       </c>
+      <c r="L21" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M21" t="n">
+        <v>60.91997184157509</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1432,9 +1599,9 @@
       <c r="G22" t="n">
         <v>60.52697371760397</v>
       </c>
-      <c r="H22" s="1" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I22" t="n">
@@ -1448,6 +1615,14 @@
       <c r="K22" t="n">
         <v>25.82971077402717</v>
       </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M22" t="n">
+        <v>93.4024621765865</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1495,6 +1670,14 @@
       <c r="K23" t="n">
         <v>10.67522732017312</v>
       </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M23" t="n">
+        <v>85.95840573217451</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1542,11 +1725,20 @@
       <c r="K24" t="n">
         <v>17.25902738173482</v>
       </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M24" t="n">
+        <v>91.68575701259354</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="H1:I1"/>
+    <mergeCell ref="L1:M1"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="F1:G1"/>

</xml_diff>

<commit_message>
results for new samples
</commit_message>
<xml_diff>
--- a/testResults/recognizersResults.xlsx
+++ b/testResults/recognizersResults.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:M62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1297,7 +1297,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NoFall/sample_00001</t>
+          <t>Fall/sample_00015</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1306,23 +1306,23 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>27.19358427488443</v>
-      </c>
-      <c r="D17" s="1" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+        <v>68.48346996749301</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>75.13097031360169</v>
-      </c>
-      <c r="F17" s="1" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+        <v>82.33549742060924</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>77.89331541789196</v>
+        <v>118.661329807118</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -1330,7 +1330,7 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>85.83645267171943</v>
+        <v>310.0720192119839</v>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
@@ -1338,7 +1338,7 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>2.609290858294099</v>
+        <v>80.63609037888719</v>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
@@ -1346,13 +1346,13 @@
         </is>
       </c>
       <c r="M17" t="n">
-        <v>83.01624438438321</v>
+        <v>-48.57439472144312</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>NoFall/sample_00002</t>
+          <t>Fall/sample_00016</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -1361,15 +1361,15 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>47.89234801910735</v>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
+        <v>19.53378462928102</v>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>41.64719072428404</v>
+        <v>48.3176779532274</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1377,37 +1377,37 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>56.39882257598806</v>
-      </c>
-      <c r="H18" s="1" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+        <v>108.2120574327766</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>167.9649363791169</v>
-      </c>
-      <c r="J18" s="1" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+        <v>247.1131095043095</v>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K18" t="n">
-        <v>51.58539717753479</v>
-      </c>
-      <c r="L18" s="1" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+        <v>129.2087197426649</v>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M18" t="n">
-        <v>29.95240519021135</v>
+        <v>14.46631422107126</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NoFall/sample_00003</t>
+          <t>Fall/sample_00017</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1416,7 +1416,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>39.43040464888713</v>
+        <v>65.42973030769349</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -1424,7 +1424,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>86.14477063161563</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1432,7 +1432,7 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>43.75768360777948</v>
+        <v>111.5409506189703</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -1440,7 +1440,7 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>47.09282872568621</v>
+        <v>364.5155172689786</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>17.50931995130208</v>
+        <v>97.86641369188938</v>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
@@ -1456,13 +1456,13 @@
         </is>
       </c>
       <c r="M19" t="n">
-        <v>97.70309957445166</v>
+        <v>-14.39733930929261</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>NoFall/sample_00004</t>
+          <t>Fall/sample_00018</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1471,7 +1471,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>8.606820544395312</v>
+        <v>60.10134764736843</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>41.59200408642722</v>
+        <v>76.69949801390406</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>64.69809565019713</v>
+        <v>101.4598087609743</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>65.29393985363899</v>
+        <v>333.1852098068209</v>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
@@ -1503,7 +1503,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>17.712211108605</v>
+        <v>66.80600050030139</v>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
@@ -1511,13 +1511,13 @@
         </is>
       </c>
       <c r="M20" t="n">
-        <v>96.05048371238728</v>
+        <v>6.651524026763187</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NoFall/sample_00005</t>
+          <t>Fall/sample_00019</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1526,15 +1526,15 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>32.67865285760173</v>
-      </c>
-      <c r="D21" s="1" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+        <v>50.93403073112643</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>51.9201425765069</v>
+        <v>48.60537284787113</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1542,15 +1542,15 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>70.63165672767941</v>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
+        <v>98.27464711686255</v>
+      </c>
+      <c r="H21" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>76.57839864030662</v>
+        <v>127.3749114280458</v>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
@@ -1558,21 +1558,21 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>12.36876507368786</v>
-      </c>
-      <c r="L21" s="1" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+        <v>66.46684603977879</v>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M21" t="n">
-        <v>60.91997184157509</v>
+        <v>5.894445578515066</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NoFall/sample_00006</t>
+          <t>Fall/sample_00020</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1581,7 +1581,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>7.744338574759364</v>
+        <v>58.25995617647428</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
@@ -1589,7 +1589,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>35.38796434509558</v>
+        <v>61.01856223661483</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>60.52697371760397</v>
+        <v>85.53564880805943</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -1605,15 +1605,15 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>120.3936226580599</v>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
+        <v>175.2186656027142</v>
+      </c>
+      <c r="J22" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K22" t="n">
-        <v>25.82971077402717</v>
+        <v>44.39495675681559</v>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
@@ -1621,13 +1621,13 @@
         </is>
       </c>
       <c r="M22" t="n">
-        <v>93.4024621765865</v>
+        <v>-4.980614092235853</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NoFall/sample_00007</t>
+          <t>Fall/sample_00021</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1636,7 +1636,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>16.70808498209217</v>
+        <v>67.18985986480266</v>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
@@ -1644,23 +1644,23 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>41.87244138638865</v>
-      </c>
-      <c r="F23" s="1" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+        <v>51.31226840567791</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>72.05970671885404</v>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
+        <v>102.2333627671665</v>
+      </c>
+      <c r="H23" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>76.6326142451359</v>
+        <v>149.6981663377549</v>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
@@ -1668,7 +1668,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>10.67522732017312</v>
+        <v>65.09704877991015</v>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
@@ -1676,62 +1676,2152 @@
         </is>
       </c>
       <c r="M23" t="n">
-        <v>85.95840573217451</v>
+        <v>-10.92273260626305</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Fall/sample_00022</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>80.8050206180052</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>139.6659226761672</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>128.9410302196652</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>431.6629704061455</v>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>85.80282202436429</v>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M24" t="n">
+        <v>-44.90808859312772</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Fall/sample_00023</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>71.7307603786589</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>70.71899472046576</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>114.3159259572131</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>248.1016842930335</v>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>76.35356943600787</v>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M25" t="n">
+        <v>-43.60033952499383</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Fall/sample_00024</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>-22.13611682351057</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>84.67276313706915</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>81.89989894257423</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>186.6829315041364</v>
+      </c>
+      <c r="J26" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>38.11662822418913</v>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M26" t="n">
+        <v>63.34507602246886</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Fall/sample_00025</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>71.2832647142241</v>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>97.87187500823801</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>106.5586670444095</v>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>579.9881912215193</v>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>84.23091516021987</v>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>-32.99128601878743</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Fall/sample_00026</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>25.8801172212624</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>62.55158948935554</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>73.95395022335745</v>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>151.5154183892844</v>
+      </c>
+      <c r="J28" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>38.62857431126842</v>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M28" t="n">
+        <v>17.17535392783295</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Fall/sample_00027</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>65.90510669402187</v>
+      </c>
+      <c r="D29" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>37.27322538214932</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>72.38305229827419</v>
+      </c>
+      <c r="H29" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>137.435915353599</v>
+      </c>
+      <c r="J29" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>40.40939050891058</v>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M29" t="n">
+        <v>64.87416900478937</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Fall/sample_00028</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>66.29601588335652</v>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>80.62319807951609</v>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>99.9074683692692</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>336.2633128273962</v>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>60.10948626890758</v>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M30" t="n">
+        <v>-24.01398321384286</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Fall/sample_00029</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>38.98039227468765</v>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>60.97447794560212</v>
+      </c>
+      <c r="F31" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>69.96028654886497</v>
+      </c>
+      <c r="H31" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>140.8773365664335</v>
+      </c>
+      <c r="J31" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>17.31431496193215</v>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M31" t="n">
+        <v>41.22966836724969</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00001</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>27.19358427488443</v>
+      </c>
+      <c r="D32" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>75.13097031360169</v>
+      </c>
+      <c r="F32" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>77.89331541789196</v>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>85.83645267171943</v>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>2.609290858294099</v>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M32" t="n">
+        <v>83.01624438438321</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00002</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>47.89234801910735</v>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>41.64719072428404</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>56.39882257598806</v>
+      </c>
+      <c r="H33" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>167.9649363791169</v>
+      </c>
+      <c r="J33" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>51.58539717753479</v>
+      </c>
+      <c r="L33" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M33" t="n">
+        <v>29.95240519021135</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00003</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>39.43040464888713</v>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>43.75768360777948</v>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>47.09282872568621</v>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>17.50931995130208</v>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M34" t="n">
+        <v>97.70309957445166</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00004</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>8.606820544395312</v>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>41.59200408642722</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>64.69809565019713</v>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>65.29393985363899</v>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
+        <v>17.712211108605</v>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M35" t="n">
+        <v>96.05048371238728</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00005</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>32.67865285760173</v>
+      </c>
+      <c r="D36" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>51.9201425765069</v>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>70.63165672767941</v>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>76.57839864030662</v>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K36" t="n">
+        <v>12.36876507368786</v>
+      </c>
+      <c r="L36" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M36" t="n">
+        <v>60.91997184157509</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00006</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>7.744338574759364</v>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>35.38796434509558</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>60.52697371760397</v>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>120.3936226580599</v>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K37" t="n">
+        <v>25.82971077402717</v>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M37" t="n">
+        <v>93.4024621765865</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00007</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>16.70808498209217</v>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>41.87244138638865</v>
+      </c>
+      <c r="F38" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>72.05970671885404</v>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>76.6326142451359</v>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K38" t="n">
+        <v>10.67522732017312</v>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M38" t="n">
+        <v>85.95840573217451</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>NoFall/sample_00008</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
         <v>22.07668311270091</v>
       </c>
-      <c r="D24" s="1" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
+      <c r="D39" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
         <v>51.74639764150002</v>
       </c>
-      <c r="F24" s="1" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
+      <c r="F39" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
         <v>73.50682347587647</v>
       </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
         <v>85.60877852981875</v>
       </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K24" t="n">
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K39" t="n">
         <v>17.25902738173482</v>
       </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="M24" t="n">
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M39" t="n">
         <v>91.68575701259354</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00009</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>-34.86282198931858</v>
+      </c>
+      <c r="D40" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>65.25700895778527</v>
+      </c>
+      <c r="F40" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>89.10919055723765</v>
+      </c>
+      <c r="H40" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>166.973354697239</v>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K40" t="n">
+        <v>14.22978210246786</v>
+      </c>
+      <c r="L40" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M40" t="n">
+        <v>13.91526693538044</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00010</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>37.41445797951537</v>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>44.37211157340168</v>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>89.57597262201709</v>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K41" t="n">
+        <v>14.05995742800313</v>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M41" t="n">
+        <v>84.88346102549325</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00011</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>32.4264707709299</v>
+      </c>
+      <c r="D42" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>62.62319198180828</v>
+      </c>
+      <c r="F42" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>85.08556928329268</v>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>101.1073652707247</v>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K42" t="n">
+        <v>35.14445419215845</v>
+      </c>
+      <c r="L42" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M42" t="n">
+        <v>15.84644323613126</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00012</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>56.14916718697047</v>
+      </c>
+      <c r="D43" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>76.88790722174474</v>
+      </c>
+      <c r="F43" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>108.3972301211737</v>
+      </c>
+      <c r="H43" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>330.6662813077434</v>
+      </c>
+      <c r="J43" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K43" t="n">
+        <v>68.75473658578858</v>
+      </c>
+      <c r="L43" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M43" t="n">
+        <v>-51.65572999174019</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00013</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>14.24489268996905</v>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>18.15924348506505</v>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>30.70185638836027</v>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>118.0161265615768</v>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K44" t="n">
+        <v>31.82152265877161</v>
+      </c>
+      <c r="L44" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M44" t="n">
+        <v>55.04298823392116</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00014</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>49.34834025125897</v>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>32.26334763179281</v>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>67.33896879616324</v>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>90.12879398060677</v>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K45" t="n">
+        <v>34.56098248463763</v>
+      </c>
+      <c r="L45" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M45" t="n">
+        <v>58.50718653014621</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00015</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>44.25506585617948</v>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>32.08521305041441</v>
+      </c>
+      <c r="F46" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>105.2704332338869</v>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>131.1383188264916</v>
+      </c>
+      <c r="J46" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K46" t="n">
+        <v>119.7335265535714</v>
+      </c>
+      <c r="L46" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M46" t="n">
+        <v>41.10839085784406</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00016</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>31.25048863107477</v>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>21.11899728653623</v>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>106.733349463466</v>
+      </c>
+      <c r="H47" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>185.0606578480502</v>
+      </c>
+      <c r="J47" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K47" t="n">
+        <v>126.8611749187042</v>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M47" t="n">
+        <v>80.8796168830559</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00017</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>11.75619035047047</v>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>30.7410751528738</v>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>30.42327050181174</v>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>123.3724464645881</v>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K48" t="n">
+        <v>10.03556828234729</v>
+      </c>
+      <c r="L48" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M48" t="n">
+        <v>61.65197714439121</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00018</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>36.45576644608872</v>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>12.19426650313514</v>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>67.7076115322115</v>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>58.04468091210849</v>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K49" t="n">
+        <v>39.0822782254108</v>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M49" t="n">
+        <v>98.32868075957093</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00019</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>49.7042879646257</v>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>1.090909712914097</v>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>64.22530959577422</v>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>80.7329408914072</v>
+      </c>
+      <c r="J50" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K50" t="n">
+        <v>50.53755466623485</v>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M50" t="n">
+        <v>91.05724086980473</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00020</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>-16.81850482037062</v>
+      </c>
+      <c r="D51" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>131.1839791560091</v>
+      </c>
+      <c r="F51" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>88.03415336358756</v>
+      </c>
+      <c r="H51" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>194.5430340819911</v>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K51" t="n">
+        <v>40.82713265082228</v>
+      </c>
+      <c r="L51" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M51" t="n">
+        <v>-1.213873597656874</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00021</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>-6.912120650875187</v>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>40.25492238877744</v>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>40.87984994336098</v>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>88.44609436085365</v>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K52" t="n">
+        <v>9.729051285607298</v>
+      </c>
+      <c r="L52" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M52" t="n">
+        <v>-5.538043413067541</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00022</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>60.35402287506971</v>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>42.67982590096265</v>
+      </c>
+      <c r="F53" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>95.69121876391071</v>
+      </c>
+      <c r="H53" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>217.1733404724765</v>
+      </c>
+      <c r="J53" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K53" t="n">
+        <v>70.73071523809016</v>
+      </c>
+      <c r="L53" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M53" t="n">
+        <v>43.98057934569032</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00023</t>
+        </is>
+      </c>
+      <c r="B54" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>62.47124416569899</v>
+      </c>
+      <c r="D54" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>58.15880894177874</v>
+      </c>
+      <c r="F54" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>105.1051048902516</v>
+      </c>
+      <c r="H54" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>175.4247675126983</v>
+      </c>
+      <c r="J54" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K54" t="n">
+        <v>70.41462670439778</v>
+      </c>
+      <c r="L54" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M54" t="n">
+        <v>-27.48712466526298</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00024</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>0.5080452789598471</v>
+      </c>
+      <c r="D55" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>53.9721745583013</v>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>51.19850539672729</v>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>85.46056048057011</v>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K55" t="n">
+        <v>36.36309976957148</v>
+      </c>
+      <c r="L55" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M55" t="n">
+        <v>77.2047751768813</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00025</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>35.61205445922448</v>
+      </c>
+      <c r="D56" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>177.3229801247136</v>
+      </c>
+      <c r="F56" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>205.9249623136563</v>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>57.42080637013869</v>
+      </c>
+      <c r="J56" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K56" t="n">
+        <v>166.2114319054999</v>
+      </c>
+      <c r="L56" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M56" t="n">
+        <v>-63.70741193018718</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00026</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>78.27110275917201</v>
+      </c>
+      <c r="D57" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>64.94593710266518</v>
+      </c>
+      <c r="F57" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>112.6942982591747</v>
+      </c>
+      <c r="H57" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>295.4353832895237</v>
+      </c>
+      <c r="J57" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K57" t="n">
+        <v>84.29540825607006</v>
+      </c>
+      <c r="L57" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M57" t="n">
+        <v>31.94143904117551</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00027</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>38.22026753990026</v>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>34.5788450054731</v>
+      </c>
+      <c r="F58" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>73.17866714675536</v>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>76.25065631689711</v>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K58" t="n">
+        <v>28.03097050420214</v>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M58" t="n">
+        <v>83.92630488854991</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00028</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>29.64148709792211</v>
+      </c>
+      <c r="D59" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>61.94086250986143</v>
+      </c>
+      <c r="F59" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>98.32760506199355</v>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>94.50948036334249</v>
+      </c>
+      <c r="J59" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K59" t="n">
+        <v>48.65784282879268</v>
+      </c>
+      <c r="L59" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M59" t="n">
+        <v>56.83755536159898</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00029</t>
+        </is>
+      </c>
+      <c r="B60" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>66.2562058531025</v>
+      </c>
+      <c r="D60" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>98.9760963448359</v>
+      </c>
+      <c r="F60" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>115.0594357244582</v>
+      </c>
+      <c r="H60" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>495.0666979760229</v>
+      </c>
+      <c r="J60" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K60" t="n">
+        <v>76.03888224551025</v>
+      </c>
+      <c r="L60" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M60" t="n">
+        <v>-23.57108187455233</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00030</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>12.01159043531782</v>
+      </c>
+      <c r="D61" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>74.06104396088782</v>
+      </c>
+      <c r="F61" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>81.85571158142037</v>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>123.004505308875</v>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K61" t="n">
+        <v>6.365086916667209</v>
+      </c>
+      <c r="L61" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M61" t="n">
+        <v>36.90527979540194</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>NoFall/sample_00031</t>
+        </is>
+      </c>
+      <c r="B62" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>57.2380380993217</v>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>21.82725799605034</v>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>59.88610443765944</v>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>129.8710253141478</v>
+      </c>
+      <c r="J62" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K62" t="n">
+        <v>57.29228128915611</v>
+      </c>
+      <c r="L62" s="1" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="M62" t="n">
+        <v>50.23991285620325</v>
       </c>
     </row>
   </sheetData>

</xml_diff>